<commit_message>
update project status testcase
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/HRM.xlsx
+++ b/src/test/resources/testdata/HRM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12765" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12765" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="2" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="102">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -181,6 +181,9 @@
     <t>Priority</t>
   </si>
   <si>
+    <t>Progress</t>
+  </si>
+  <si>
     <t>This is auto test1</t>
   </si>
   <si>
@@ -205,6 +208,9 @@
     <t>Highest</t>
   </si>
   <si>
+    <t>39</t>
+  </si>
+  <si>
     <t>This is auto test2</t>
   </si>
   <si>
@@ -226,6 +232,9 @@
     <t>Low</t>
   </si>
   <si>
+    <t>100</t>
+  </si>
+  <si>
     <t>This is auto test3</t>
   </si>
   <si>
@@ -247,6 +256,9 @@
     <t>Normal</t>
   </si>
   <si>
+    <t>50</t>
+  </si>
+  <si>
     <t>This is auto test4</t>
   </si>
   <si>
@@ -262,6 +274,9 @@
     <t>09-09-2029</t>
   </si>
   <si>
+    <t>68</t>
+  </si>
+  <si>
     <t>This is auto test5</t>
   </si>
   <si>
@@ -277,6 +292,9 @@
     <t>09-09-2030</t>
   </si>
   <si>
+    <t>23</t>
+  </si>
+  <si>
     <t>TC06</t>
   </si>
   <si>
@@ -296,6 +314,9 @@
   </si>
   <si>
     <t>High</t>
+  </si>
+  <si>
+    <t>9</t>
   </si>
   <si>
     <t>Endate</t>
@@ -309,10 +330,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -344,7 +365,99 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -358,57 +471,25 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -419,66 +500,6 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="34">
     <fill>
@@ -495,187 +516,187 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -686,6 +707,71 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -708,30 +794,6 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
@@ -745,59 +807,18 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -807,130 +828,130 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1540,7 +1561,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="6"/>
   <cols>
     <col min="1" max="1" width="12.5619047619048" customWidth="1"/>
@@ -1553,7 +1574,7 @@
     <col min="8" max="8" width="12.6190476190476" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1581,179 +1602,200 @@
       <c r="I1" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>62</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>70</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="H4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+        <v>78</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" s="3" t="s">
         <v>35</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="H5" t="s">
         <v>77</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="F5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="H5" t="s">
-        <v>74</v>
-      </c>
       <c r="I5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+        <v>70</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" s="3" t="s">
         <v>41</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="H6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
+        <v>62</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" s="3" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="H7" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="I7" t="s">
-        <v>92</v>
+        <v>98</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1784,10 +1826,10 @@
         <v>48</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>50</v>
@@ -1798,7 +1840,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1806,7 +1848,7 @@
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1814,7 +1856,7 @@
         <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1822,7 +1864,7 @@
         <v>35</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1830,15 +1872,15 @@
         <v>41</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="3" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update testcase add file project
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/HRM.xlsx
+++ b/src/test/resources/testdata/HRM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="13035" activeTab="3"/>
+    <workbookView windowWidth="28800" windowHeight="12765" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="2" r:id="rId1"/>
@@ -369,10 +369,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -397,6 +397,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
@@ -404,7 +411,31 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -418,11 +449,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -433,16 +486,32 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -456,62 +525,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -524,21 +539,6 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="35">
     <fill>
@@ -561,13 +561,85 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -579,85 +651,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -669,73 +717,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -752,6 +752,30 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -769,8 +793,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -805,26 +829,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -843,160 +852,151 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="21" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="24" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>

</xml_diff>

<commit_message>
change data test in excel
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/HRM.xlsx
+++ b/src/test/resources/testdata/HRM.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="13035" activeTab="4"/>
+    <workbookView windowWidth="28800" windowHeight="13035" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="2" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="132">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -197,172 +197,160 @@
     <t>An Nguyen</t>
   </si>
   <si>
+    <t>04-11-2025</t>
+  </si>
+  <si>
+    <t>Run auto test</t>
+  </si>
+  <si>
+    <t>09-09-2026</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Highest</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>Image test</t>
+  </si>
+  <si>
+    <t>This is auto project2</t>
+  </si>
+  <si>
+    <t>Alex Pham</t>
+  </si>
+  <si>
+    <t>05-09-2025</t>
+  </si>
+  <si>
+    <t>01-11-2026</t>
+  </si>
+  <si>
+    <t>09-09-2027</t>
+  </si>
+  <si>
+    <t>On Hold</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>This is auto project3</t>
+  </si>
+  <si>
+    <t>05-10-2027</t>
+  </si>
+  <si>
+    <t>20-12-2027</t>
+  </si>
+  <si>
+    <t>09-09-2028</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>This is auto project4</t>
+  </si>
+  <si>
+    <t>05-10-2028</t>
+  </si>
+  <si>
+    <t>20-12-2028</t>
+  </si>
+  <si>
+    <t>09-09-2029</t>
+  </si>
+  <si>
+    <t>68</t>
+  </si>
+  <si>
+    <t>This is auto project5</t>
+  </si>
+  <si>
+    <t>05-10-2029</t>
+  </si>
+  <si>
+    <t>20-12-2029</t>
+  </si>
+  <si>
+    <t>09-09-2030</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>Title task</t>
+  </si>
+  <si>
+    <t>Endate</t>
+  </si>
+  <si>
+    <t>Project</t>
+  </si>
+  <si>
+    <t>This is auto task1</t>
+  </si>
+  <si>
     <t>01-01-2025</t>
   </si>
   <si>
+    <t>20-12-2025</t>
+  </si>
+  <si>
+    <t>This is a test task with more than sixty characters to meet the requirement.</t>
+  </si>
+  <si>
+    <t>This is auto task2</t>
+  </si>
+  <si>
     <t>01-01-2026</t>
   </si>
   <si>
-    <t>Run auto test</t>
-  </si>
-  <si>
-    <t>09-09-2026</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>Highest</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>Image test</t>
-  </si>
-  <si>
-    <t>This is auto project2</t>
-  </si>
-  <si>
-    <t>Alex Pham</t>
-  </si>
-  <si>
-    <t>05-09-2025</t>
-  </si>
-  <si>
-    <t>01-11-2026</t>
-  </si>
-  <si>
-    <t>09-09-2027</t>
-  </si>
-  <si>
-    <t>On Hold</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>This is auto project3</t>
-  </si>
-  <si>
-    <t>05-10-2027</t>
-  </si>
-  <si>
-    <t>20-12-2027</t>
-  </si>
-  <si>
-    <t>09-09-2028</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>Normal</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>This is auto project4</t>
-  </si>
-  <si>
-    <t>05-10-2028</t>
-  </si>
-  <si>
-    <t>20-12-2028</t>
-  </si>
-  <si>
-    <t>09-09-2029</t>
-  </si>
-  <si>
-    <t>68</t>
-  </si>
-  <si>
-    <t>This is auto project5</t>
-  </si>
-  <si>
-    <t>05-10-2029</t>
-  </si>
-  <si>
-    <t>20-12-2029</t>
-  </si>
-  <si>
-    <t>09-09-2030</t>
-  </si>
-  <si>
-    <t>23</t>
+    <t>20-12-2026</t>
+  </si>
+  <si>
+    <t>This is auto task3</t>
+  </si>
+  <si>
+    <t>01-01-2027</t>
+  </si>
+  <si>
+    <t>This is auto task4</t>
+  </si>
+  <si>
+    <t>01-01-2028</t>
+  </si>
+  <si>
+    <t>This is auto task5</t>
+  </si>
+  <si>
+    <t>01-01-2029</t>
   </si>
   <si>
     <t>TC06</t>
   </si>
   <si>
-    <t>This is auto project6</t>
-  </si>
-  <si>
-    <t>05-10-2025</t>
+    <t>This is auto task6</t>
+  </si>
+  <si>
+    <t>01-01-2030</t>
   </si>
   <si>
     <t>20-12-2030</t>
-  </si>
-  <si>
-    <t>09-09-2031</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>Title task</t>
-  </si>
-  <si>
-    <t>Endate</t>
-  </si>
-  <si>
-    <t>Project</t>
-  </si>
-  <si>
-    <t>This is auto task1</t>
-  </si>
-  <si>
-    <t>20-12-2025</t>
-  </si>
-  <si>
-    <t>This is a test task with more than sixty characters to meet the requirement.</t>
-  </si>
-  <si>
-    <t>This is auto task2</t>
-  </si>
-  <si>
-    <t>20-12-2026</t>
-  </si>
-  <si>
-    <t>This is auto task3</t>
-  </si>
-  <si>
-    <t>01-01-2027</t>
-  </si>
-  <si>
-    <t>This is auto task4</t>
-  </si>
-  <si>
-    <t>01-01-2028</t>
-  </si>
-  <si>
-    <t>This is auto task5</t>
-  </si>
-  <si>
-    <t>01-01-2029</t>
-  </si>
-  <si>
-    <t>This is auto task6</t>
-  </si>
-  <si>
-    <t>01-01-2030</t>
   </si>
   <si>
     <t>Username_admin</t>
@@ -469,7 +457,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -483,14 +471,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -501,14 +489,6 @@
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -528,24 +508,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -559,8 +524,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -568,6 +556,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -589,20 +584,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="39">
     <fill>
@@ -649,12 +637,174 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -667,169 +817,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -843,26 +831,26 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -896,23 +884,32 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color rgb="FF7F7F7F"/>
       </left>
       <right style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color rgb="FF7F7F7F"/>
       </right>
       <top style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color rgb="FF7F7F7F"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -931,19 +928,10 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -961,130 +949,130 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="27" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="28" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="35" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1704,8 +1692,8 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="6"/>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="12.5619047619048" customWidth="1"/>
     <col min="2" max="2" width="19.8666666666667" customWidth="1"/>
@@ -1769,25 +1757,25 @@
         <v>59</v>
       </c>
       <c r="E2" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="F2" t="s">
         <v>60</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="H2" t="s">
         <v>62</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>63</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="J2" s="16" t="s">
+      <c r="K2" t="s">
         <v>65</v>
-      </c>
-      <c r="K2" t="s">
-        <v>66</v>
       </c>
       <c r="L2" t="s">
         <v>23</v>
@@ -1798,34 +1786,34 @@
         <v>6</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D3" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="E3" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="F3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G3" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="F3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G3" s="16" t="s">
+      <c r="H3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>72</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="J3" s="16" t="s">
-        <v>74</v>
-      </c>
       <c r="K3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L3" t="s">
         <v>23</v>
@@ -1836,34 +1824,34 @@
         <v>8</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D4" s="14" t="s">
+      <c r="E4" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="F4" t="s">
-        <v>61</v>
-      </c>
-      <c r="G4" s="16" t="s">
+      <c r="H4" t="s">
         <v>78</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>79</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="J4" s="16" t="s">
-        <v>81</v>
-      </c>
       <c r="K4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L4" t="s">
         <v>23</v>
@@ -1874,34 +1862,34 @@
         <v>35</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C5" t="s">
         <v>58</v>
       </c>
       <c r="D5" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="F5" t="s">
-        <v>61</v>
-      </c>
-      <c r="G5" s="16" t="s">
+      <c r="H5" t="s">
+        <v>78</v>
+      </c>
+      <c r="I5" t="s">
+        <v>72</v>
+      </c>
+      <c r="J5" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="H5" t="s">
-        <v>79</v>
-      </c>
-      <c r="I5" t="s">
-        <v>73</v>
-      </c>
-      <c r="J5" s="16" t="s">
-        <v>86</v>
-      </c>
       <c r="K5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L5" t="s">
         <v>23</v>
@@ -1912,74 +1900,36 @@
         <v>41</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D6" s="14" t="s">
+      <c r="E6" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="F6" t="s">
-        <v>61</v>
-      </c>
-      <c r="G6" s="16" t="s">
+      <c r="H6" t="s">
+        <v>62</v>
+      </c>
+      <c r="I6" t="s">
+        <v>63</v>
+      </c>
+      <c r="J6" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="H6" t="s">
-        <v>63</v>
-      </c>
-      <c r="I6" t="s">
-        <v>64</v>
-      </c>
-      <c r="J6" s="16" t="s">
-        <v>91</v>
-      </c>
       <c r="K6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>95</v>
-      </c>
-      <c r="F7" t="s">
-        <v>61</v>
-      </c>
-      <c r="G7" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="H7" t="s">
-        <v>79</v>
-      </c>
-      <c r="I7" t="s">
-        <v>97</v>
-      </c>
-      <c r="J7" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="K7" t="s">
-        <v>66</v>
-      </c>
-      <c r="L7" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2007,16 +1957,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>48</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>50</v>
@@ -2028,19 +1978,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>59</v>
+        <v>95</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2048,19 +1998,19 @@
         <v>6</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>60</v>
+        <v>99</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E3" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="F3" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2068,19 +2018,19 @@
         <v>8</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E4" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2088,19 +2038,19 @@
         <v>35</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E5" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="F5" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2108,39 +2058,39 @@
         <v>41</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E6" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="F6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="E7" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="F7" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2168,10 +2118,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>10</v>
@@ -2180,10 +2130,10 @@
         <v>11</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>13</v>
@@ -2192,37 +2142,37 @@
         <v>14</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="L1" s="5" t="s">
         <v>46</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>47</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="S1" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="T1" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -2236,10 +2186,10 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F2" s="16" t="s">
         <v>5</v>
@@ -2251,40 +2201,40 @@
         <v>27</v>
       </c>
       <c r="I2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="J2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="K2" t="s">
         <v>23</v>
       </c>
       <c r="L2" t="s">
+        <v>127</v>
+      </c>
+      <c r="M2" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="N2" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="O2" t="s">
+        <v>130</v>
+      </c>
+      <c r="P2" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q2" t="s">
         <v>131</v>
       </c>
-      <c r="M2" s="16" t="s">
-        <v>132</v>
-      </c>
-      <c r="N2" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="O2" t="s">
-        <v>134</v>
-      </c>
-      <c r="P2" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>135</v>
-      </c>
       <c r="R2" s="16" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="S2" s="16" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="T2" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>